<commit_message>
fix(web): ADI-01 version consolidada (22 fuentes) + enlace clickeable en artefactos
- Artefactos re-extraidos del workbook actual (no bak): ADI-01 pasa de 34 a 22 fuentes; ADI-03/07 mas completos.

- Grid muestra el enlace (hipervinculo a Drive) como link clickeable (gen_artefactos captura cell.hyperlink).

- fuentes_institucionales recargada desde ADI-01 de 22 + columna 'enlace' (schema.sql + Prisma). Nuevas renumeradas F-23/24/25.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-04.xlsx
+++ b/client/public/artefactos/ADI-04.xlsx
@@ -271,7 +271,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -455,11 +455,44 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -608,6 +641,14 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>

<commit_message>
ADI-04: columnas de análisis (Vacíos/dispersión, Observaciones modelo conceptual) sin marca * (su naturaleza inferida se sobreentiende)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-04.xlsx
+++ b/client/public/artefactos/ADI-04.xlsx
@@ -558,12 +558,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>26 fuente(s) de datos asociada(s); 25 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Aporte' aparece en 1 fuentes del dominio. *</t>
+          <t>26 fuente(s) de datos asociada(s); 25 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Aporte' aparece en 1 fuentes del dominio.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Aporte' (presente en 1 de 1 fuentes con catálogo). Entidades relevantes: Aporte, Persona, Documento, Asegurado/Afiliado. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Aporte' (presente en 1 de 1 fuentes con catálogo). Entidades relevantes: Aporte, Persona, Documento, Asegurado/Afiliado. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -626,12 +626,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>11 fuente(s) de datos asociada(s); 3 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 8 fuentes del dominio. Solapamiento: Documento, Solicitud, Aporte compartida(s) por ≥2 fuentes (posible duplicidad). *</t>
+          <t>11 fuente(s) de datos asociada(s); 3 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 8 fuentes del dominio. Solapamiento: Documento, Solicitud, Aporte compartida(s) por ≥2 fuentes (posible duplicidad).</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 8 de 8 fuentes con catálogo). Entidades relevantes: Documento, Solicitud, Aporte, Persona. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Documento' (presente en 8 de 8 fuentes con catálogo). Entidades relevantes: Documento, Solicitud, Aporte, Persona. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -694,12 +694,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>1 fuente(s) de datos asociada(s). Dispersión: la entidad 'Documento' aparece en 1 fuentes del dominio. *</t>
+          <t>1 fuente(s) de datos asociada(s). Dispersión: la entidad 'Documento' aparece en 1 fuentes del dominio.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 1 de 1 fuentes con catálogo). Entidades relevantes: Documento, Recaudación/Pago, Asegurado/Afiliado, Persona. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Documento' (presente en 1 de 1 fuentes con catálogo). Entidades relevantes: Documento, Recaudación/Pago, Asegurado/Afiliado, Persona. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>3 fuente(s) de datos asociada(s); 1 proceso(s) del dominio sin sistema (vacío funcional). Dispersión: la entidad 'Aporte' aparece en 3 fuentes del dominio. Solapamiento: Aporte, Persona, Documento compartida(s) por ≥2 fuentes (posible duplicidad). *</t>
+          <t>3 fuente(s) de datos asociada(s); 1 proceso(s) del dominio sin sistema (vacío funcional). Dispersión: la entidad 'Aporte' aparece en 3 fuentes del dominio. Solapamiento: Aporte, Persona, Documento compartida(s) por ≥2 fuentes (posible duplicidad).</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Aporte' (presente en 3 de 3 fuentes con catálogo). Entidades relevantes: Aporte, Persona, Documento, Asegurado/Afiliado. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Aporte' (presente en 3 de 3 fuentes con catálogo). Entidades relevantes: Aporte, Persona, Documento, Asegurado/Afiliado. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>10 fuente(s) de datos asociada(s); 1 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 9 fuentes del dominio. Solapamiento: Documento, Solicitud, Aporte compartida(s) por ≥2 fuentes (posible duplicidad). *</t>
+          <t>10 fuente(s) de datos asociada(s); 1 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 9 fuentes del dominio. Solapamiento: Documento, Solicitud, Aporte compartida(s) por ≥2 fuentes (posible duplicidad).</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 9 de 9 fuentes con catálogo). Entidades relevantes: Documento, Solicitud, Aporte, Expediente/Trámite. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Documento' (presente en 9 de 9 fuentes con catálogo). Entidades relevantes: Documento, Solicitud, Aporte, Expediente/Trámite. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -902,12 +902,12 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>82 fuente(s) de datos asociada(s); 60 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 21 fuentes del dominio. Solapamiento: Documento, Expediente/Trámite, Persona compartida(s) por ≥2 fuentes (posible duplicidad). *</t>
+          <t>82 fuente(s) de datos asociada(s); 60 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 21 fuentes del dominio. Solapamiento: Documento, Expediente/Trámite, Persona compartida(s) por ≥2 fuentes (posible duplicidad).</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 21 de 22 fuentes con catálogo). Entidades relevantes: Documento, Expediente/Trámite, Persona, Solicitud. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Documento' (presente en 21 de 22 fuentes con catálogo). Entidades relevantes: Documento, Expediente/Trámite, Persona, Solicitud. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>9 fuente(s) de datos asociada(s); 2 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Aporte' aparece en 7 fuentes del dominio. Solapamiento: Aporte, Persona, Documento compartida(s) por ≥2 fuentes (posible duplicidad). *</t>
+          <t>9 fuente(s) de datos asociada(s); 2 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Aporte' aparece en 7 fuentes del dominio. Solapamiento: Aporte, Persona, Documento compartida(s) por ≥2 fuentes (posible duplicidad).</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Aporte' (presente en 7 de 7 fuentes con catálogo). Entidades relevantes: Aporte, Persona, Documento, Asegurado/Afiliado. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Aporte' (presente en 7 de 7 fuentes con catálogo). Entidades relevantes: Aporte, Persona, Documento, Asegurado/Afiliado. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -1046,12 +1046,12 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>50 fuente(s) de datos asociada(s); 47 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Aporte' aparece en 3 fuentes del dominio. Solapamiento: Aporte, Documento, Persona compartida(s) por ≥2 fuentes (posible duplicidad). *</t>
+          <t>50 fuente(s) de datos asociada(s); 47 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Aporte' aparece en 3 fuentes del dominio. Solapamiento: Aporte, Documento, Persona compartida(s) por ≥2 fuentes (posible duplicidad).</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Aporte' (presente en 3 de 3 fuentes con catálogo). Entidades relevantes: Aporte, Documento, Persona, Expediente/Trámite. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Aporte' (presente en 3 de 3 fuentes con catálogo). Entidades relevantes: Aporte, Documento, Persona, Expediente/Trámite. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -1118,12 +1118,12 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>17 fuente(s) de datos asociada(s); 8 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 9 fuentes del dominio. Solapamiento: Documento, Expediente/Trámite, Notificación compartida(s) por ≥2 fuentes (posible duplicidad). *</t>
+          <t>17 fuente(s) de datos asociada(s); 8 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 9 fuentes del dominio. Solapamiento: Documento, Expediente/Trámite, Notificación compartida(s) por ≥2 fuentes (posible duplicidad).</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 9 de 9 fuentes con catálogo). Entidades relevantes: Documento, Expediente/Trámite, Notificación, Persona. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Documento' (presente en 9 de 9 fuentes con catálogo). Entidades relevantes: Documento, Expediente/Trámite, Notificación, Persona. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -1190,12 +1190,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>73 fuente(s) de datos asociada(s); 56 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 16 fuentes del dominio. Solapamiento: Documento, Aporte, Persona compartida(s) por ≥2 fuentes (posible duplicidad). *</t>
+          <t>73 fuente(s) de datos asociada(s); 56 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 16 fuentes del dominio. Solapamiento: Documento, Aporte, Persona compartida(s) por ≥2 fuentes (posible duplicidad).</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 16 de 17 fuentes con catálogo). Entidades relevantes: Documento, Aporte, Persona, Solicitud. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Documento' (presente en 16 de 17 fuentes con catálogo). Entidades relevantes: Documento, Aporte, Persona, Solicitud. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -1238,12 +1238,12 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Sin fuentes de datos asociadas al dominio (vacío total). *</t>
+          <t>Sin fuentes de datos asociadas al dominio (vacío total).</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Sin entidades detectadas (fuentes sin catálogo físico o dominio no misional). *</t>
+          <t>Sin entidades detectadas (fuentes sin catálogo físico o dominio no misional).</t>
         </is>
       </c>
     </row>
@@ -1310,12 +1310,12 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>4 fuente(s) de datos asociada(s); 2 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 2 fuentes del dominio. Solapamiento: Documento, Persona, Solicitud compartida(s) por ≥2 fuentes (posible duplicidad). *</t>
+          <t>4 fuente(s) de datos asociada(s); 2 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 2 fuentes del dominio. Solapamiento: Documento, Persona, Solicitud compartida(s) por ≥2 fuentes (posible duplicidad).</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 2 de 2 fuentes con catálogo). Entidades relevantes: Documento, Persona, Solicitud, Expediente/Trámite. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Documento' (presente en 2 de 2 fuentes con catálogo). Entidades relevantes: Documento, Persona, Solicitud, Expediente/Trámite. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -1378,12 +1378,12 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>6 fuente(s) de datos asociada(s); 5 sin catálogo de entidades (cobertura del modelo parcial); 1 proceso(s) del dominio sin sistema (vacío funcional). Dispersión: la entidad 'Aporte' aparece en 1 fuentes del dominio. *</t>
+          <t>6 fuente(s) de datos asociada(s); 5 sin catálogo de entidades (cobertura del modelo parcial); 1 proceso(s) del dominio sin sistema (vacío funcional). Dispersión: la entidad 'Aporte' aparece en 1 fuentes del dominio.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Aporte' (presente en 1 de 1 fuentes con catálogo). Entidades relevantes: Aporte, Asegurado/Afiliado, Documento, Planilla. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Aporte' (presente en 1 de 1 fuentes con catálogo). Entidades relevantes: Aporte, Asegurado/Afiliado, Documento, Planilla. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -1446,12 +1446,12 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>1 fuente(s) de datos asociada(s). Dispersión: la entidad 'Documento' aparece en 1 fuentes del dominio. *</t>
+          <t>1 fuente(s) de datos asociada(s). Dispersión: la entidad 'Documento' aparece en 1 fuentes del dominio.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 1 de 1 fuentes con catálogo). Entidades relevantes: Documento, Recaudación/Pago, Expediente/Trámite, Persona. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC). *</t>
+          <t>Aporta principalmente la entidad 'Documento' (presente en 1 de 1 fuentes con catálogo). Entidades relevantes: Documento, Recaudación/Pago, Expediente/Trámite, Persona. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ADI-04: texto de análisis replanteado (fragmentación estructural + brecha de documentación, sin claim de duplicación de datos)
- Vacíos/dispersión y Obs. modelo conceptual: narrativa honesta por dominio desde metadata
  (entidad fragmentada en N BD + % columnas comentadas), condicionada a la dispersión real
  (fragmentación si entidad en ≥2 BD; baja cobertura de catálogo si no). Sin afirmar duplicación
  de registros (no hay acceso a datos). analisis_dominio_adi04.py

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-04.xlsx
+++ b/client/public/artefactos/ADI-04.xlsx
@@ -558,12 +558,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>26 fuente(s) de datos asociada(s); 25 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Aporte' aparece en 1 fuentes del dominio.</t>
+          <t>De 26 fuentes del dominio, solo 1 con catálogo de entidades documentado (cobertura del modelo parcial). El 15% de las columnas tiene comentarios, por lo que la documentación del dato es limitada.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Aporte' (presente en 1 de 1 fuentes con catálogo). Entidades relevantes: Aporte, Persona, Documento, Asegurado/Afiliado. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>La entidad predominante del dominio es 'Aporte'. Conviene ampliar el catálogo de las 25 fuentes sin documentar para el modelado. Correspondencia con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -626,12 +626,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>11 fuente(s) de datos asociada(s); 3 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 8 fuentes del dominio. Solapamiento: Documento, Solicitud, Aporte compartida(s) por ≥2 fuentes (posible duplicidad).</t>
+          <t>Las entidades core del dominio están fragmentadas entre varias de sus 11 fuentes ('Documento' en 8 BD, 'Solicitud' en 8 BD, 'Aporte' en 8 BD, 'Persona' en 8 BD), sin un maestro único consolidado. Además, solo el 55% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 8 de 8 fuentes con catálogo). Entidades relevantes: Documento, Solicitud, Aporte, Persona. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>'Documento' es la entidad más transversal del dominio (presente en 8 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Solicitud, Aporte para reducir la fragmentación. Debe mejorarse la documentación (55% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -694,12 +694,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>1 fuente(s) de datos asociada(s). Dispersión: la entidad 'Documento' aparece en 1 fuentes del dominio.</t>
+          <t>El dominio se concentra en 1 fuente, sin fragmentación de entidades entre fuentes. El 45% de las columnas tiene comentarios; conviene mejorar la documentación del dato.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 1 de 1 fuentes con catálogo). Entidades relevantes: Documento, Recaudación/Pago, Asegurado/Afiliado, Persona. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>La entidad predominante del dominio es 'Documento'. Conviene mejorar la documentación (45% columnas comentadas) para el modelado. Correspondencia con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>3 fuente(s) de datos asociada(s); 1 proceso(s) del dominio sin sistema (vacío funcional). Dispersión: la entidad 'Aporte' aparece en 3 fuentes del dominio. Solapamiento: Aporte, Persona, Documento compartida(s) por ≥2 fuentes (posible duplicidad).</t>
+          <t>Las entidades core del dominio están fragmentadas entre varias de sus 3 fuentes ('Aporte' en 3 BD, 'Persona' en 3 BD, 'Documento' en 3 BD, 'Asegurado/Afiliado' en 3 BD), sin un maestro único consolidado. Además, solo el 22% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Aporte' (presente en 3 de 3 fuentes con catálogo). Entidades relevantes: Aporte, Persona, Documento, Asegurado/Afiliado. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>'Aporte' es la entidad más transversal del dominio (presente en 3 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Persona, Documento para reducir la fragmentación. Debe mejorarse la documentación (22% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>10 fuente(s) de datos asociada(s); 1 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 9 fuentes del dominio. Solapamiento: Documento, Solicitud, Aporte compartida(s) por ≥2 fuentes (posible duplicidad).</t>
+          <t>Las entidades core del dominio están fragmentadas entre varias de sus 10 fuentes ('Documento' en 9 BD, 'Solicitud' en 9 BD, 'Aporte' en 9 BD, 'Expediente/Trámite' en 9 BD), sin un maestro único consolidado. Además, solo el 40% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 9 de 9 fuentes con catálogo). Entidades relevantes: Documento, Solicitud, Aporte, Expediente/Trámite. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>'Documento' es la entidad más transversal del dominio (presente en 9 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Solicitud, Aporte para reducir la fragmentación. Debe mejorarse la documentación (40% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -902,12 +902,12 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>82 fuente(s) de datos asociada(s); 60 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 21 fuentes del dominio. Solapamiento: Documento, Expediente/Trámite, Persona compartida(s) por ≥2 fuentes (posible duplicidad).</t>
+          <t>Las entidades core del dominio están fragmentadas entre varias de sus 82 fuentes ('Documento' en 21 BD, 'Expediente/Trámite' en 21 BD, 'Persona' en 20 BD, 'Solicitud' en 20 BD), sin un maestro único consolidado. Además, solo el 34% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 21 de 22 fuentes con catálogo). Entidades relevantes: Documento, Expediente/Trámite, Persona, Solicitud. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>'Documento' es la entidad más transversal del dominio (presente en 21 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Expediente/Trámite, Persona para reducir la fragmentación. Debe mejorarse la documentación (34% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>9 fuente(s) de datos asociada(s); 2 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Aporte' aparece en 7 fuentes del dominio. Solapamiento: Aporte, Persona, Documento compartida(s) por ≥2 fuentes (posible duplicidad).</t>
+          <t>Las entidades core del dominio están fragmentadas entre varias de sus 9 fuentes ('Aporte' en 7 BD, 'Persona' en 7 BD, 'Documento' en 7 BD, 'Asegurado/Afiliado' en 7 BD), sin un maestro único consolidado. Además, solo el 23% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Aporte' (presente en 7 de 7 fuentes con catálogo). Entidades relevantes: Aporte, Persona, Documento, Asegurado/Afiliado. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>'Aporte' es la entidad más transversal del dominio (presente en 7 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Persona, Documento para reducir la fragmentación. Debe mejorarse la documentación (23% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -1046,12 +1046,12 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>50 fuente(s) de datos asociada(s); 47 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Aporte' aparece en 3 fuentes del dominio. Solapamiento: Aporte, Documento, Persona compartida(s) por ≥2 fuentes (posible duplicidad).</t>
+          <t>Las entidades core del dominio están fragmentadas entre varias de sus 50 fuentes ('Aporte' en 3 BD, 'Documento' en 3 BD, 'Persona' en 3 BD, 'Expediente/Trámite' en 3 BD), sin un maestro único consolidado. Además, solo el 57% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Aporte' (presente en 3 de 3 fuentes con catálogo). Entidades relevantes: Aporte, Documento, Persona, Expediente/Trámite. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>'Aporte' es la entidad más transversal del dominio (presente en 3 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Documento, Persona para reducir la fragmentación. Debe mejorarse la documentación (57% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -1118,12 +1118,12 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>17 fuente(s) de datos asociada(s); 8 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 9 fuentes del dominio. Solapamiento: Documento, Expediente/Trámite, Notificación compartida(s) por ≥2 fuentes (posible duplicidad).</t>
+          <t>Las entidades core del dominio están fragmentadas entre varias de sus 17 fuentes ('Documento' en 9 BD, 'Expediente/Trámite' en 9 BD, 'Notificación' en 9 BD, 'Persona' en 8 BD), sin un maestro único consolidado. Además, solo el 48% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 9 de 9 fuentes con catálogo). Entidades relevantes: Documento, Expediente/Trámite, Notificación, Persona. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>'Documento' es la entidad más transversal del dominio (presente en 9 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Expediente/Trámite, Notificación para reducir la fragmentación. Debe mejorarse la documentación (48% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -1190,12 +1190,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>73 fuente(s) de datos asociada(s); 56 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 16 fuentes del dominio. Solapamiento: Documento, Aporte, Persona compartida(s) por ≥2 fuentes (posible duplicidad).</t>
+          <t>Las entidades core del dominio están fragmentadas entre varias de sus 73 fuentes ('Documento' en 16 BD, 'Aporte' en 15 BD, 'Persona' en 15 BD, 'Solicitud' en 15 BD), sin un maestro único consolidado. Además, solo el 24% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 16 de 17 fuentes con catálogo). Entidades relevantes: Documento, Aporte, Persona, Solicitud. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>'Documento' es la entidad más transversal del dominio (presente en 16 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Aporte, Persona para reducir la fragmentación. Debe mejorarse la documentación (24% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -1238,12 +1238,12 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Sin fuentes de datos asociadas al dominio (vacío total).</t>
+          <t>Sin fuentes de datos asociadas en el inventario: vacío total (no hay sistemas ni BD mapeadas).</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Sin entidades detectadas (fuentes sin catálogo físico o dominio no misional).</t>
+          <t>Sin entidades detectadas (fuentes sin catálogo o dominio no misional); requiere identificar sus sistemas de soporte para el modelado.</t>
         </is>
       </c>
     </row>
@@ -1310,12 +1310,12 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>4 fuente(s) de datos asociada(s); 2 sin catálogo de entidades (cobertura del modelo parcial). Dispersión: la entidad 'Documento' aparece en 2 fuentes del dominio. Solapamiento: Documento, Persona, Solicitud compartida(s) por ≥2 fuentes (posible duplicidad).</t>
+          <t>Las entidades core del dominio están fragmentadas entre varias de sus 4 fuentes ('Documento' en 2 BD, 'Persona' en 2 BD, 'Solicitud' en 2 BD, 'Expediente/Trámite' en 2 BD), sin un maestro único consolidado. Además, solo el 46% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 2 de 2 fuentes con catálogo). Entidades relevantes: Documento, Persona, Solicitud, Expediente/Trámite. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>'Documento' es la entidad más transversal del dominio (presente en 2 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Persona, Solicitud para reducir la fragmentación. Debe mejorarse la documentación (46% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -1378,12 +1378,12 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>6 fuente(s) de datos asociada(s); 5 sin catálogo de entidades (cobertura del modelo parcial); 1 proceso(s) del dominio sin sistema (vacío funcional). Dispersión: la entidad 'Aporte' aparece en 1 fuentes del dominio.</t>
+          <t>De 6 fuentes del dominio, solo 1 con catálogo de entidades documentado (cobertura del modelo parcial). El 81% de las columnas tiene comentarios, por lo que la documentación del dato es limitada.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Aporte' (presente en 1 de 1 fuentes con catálogo). Entidades relevantes: Aporte, Asegurado/Afiliado, Documento, Planilla. 'Aporte' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>La entidad predominante del dominio es 'Aporte'. Conviene ampliar el catálogo de las 5 fuentes sin documentar para el modelado. Correspondencia con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>
@@ -1446,12 +1446,12 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>1 fuente(s) de datos asociada(s). Dispersión: la entidad 'Documento' aparece en 1 fuentes del dominio.</t>
+          <t>El dominio se concentra en 1 fuente, sin fragmentación de entidades entre fuentes. El 66% de las columnas tiene comentarios; conviene mejorar la documentación del dato.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Aporta principalmente la entidad 'Documento' (presente en 1 de 1 fuentes con catálogo). Entidades relevantes: Documento, Recaudación/Pago, Expediente/Trámite, Persona. 'Documento' candidata a entidad maestra del modelo conceptual BDI. Alineación con el SIIP pendiente (dominios de datos aún no definidos en el MC).</t>
+          <t>La entidad predominante del dominio es 'Documento'. Conviene mejorar la documentación (66% columnas comentadas) para el modelado. Correspondencia con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ADI-04: severidad por percentil de documentación en Vacíos/dispersión; Obs. modelo conceptual = solo entidades que aporta
- Vacíos/dispersión: prefijo 'Severidad {Crítica..Mínima} (N% documentado)' por percentil del % de
  columnas comentadas (0%=más severa → 100%=favorable); aclarado 'estructura física catalogada'
- Observaciones modelo conceptual: lista únicamente las entidades que el dominio aporta

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-04.xlsx
+++ b/client/public/artefactos/ADI-04.xlsx
@@ -558,12 +558,12 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>De 26 fuentes del dominio, solo 1 con catálogo de entidades documentado (cobertura del modelo parcial). El 15% de las columnas tiene comentarios, por lo que la documentación del dato es limitada.</t>
+          <t>Severidad Crítica (15% documentado): de 26 fuentes del dominio, solo 1 tiene su estructura física catalogada (cobertura del modelo parcial); el 15% de las columnas tiene comentarios.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>La entidad predominante del dominio es 'Aporte'. Conviene ampliar el catálogo de las 25 fuentes sin documentar para el modelado. Correspondencia con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Aporte, Persona, Documento, Asegurado/Afiliado, Empleador/Aportante, Recaudación/Pago, Pensión/Pensionista, SCTR, Expediente/Trámite, Planilla, Solicitud, Beneficiario, Resolución, Derecho previsional, Prestación/Beneficio, Notificación, Fiscalización, Inversión/FCR.</t>
         </is>
       </c>
     </row>
@@ -626,12 +626,12 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Las entidades core del dominio están fragmentadas entre varias de sus 11 fuentes ('Documento' en 8 BD, 'Solicitud' en 8 BD, 'Aporte' en 8 BD, 'Persona' en 8 BD), sin un maestro único consolidado. Además, solo el 55% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
+          <t>Severidad Baja (55% documentado): las entidades core están fragmentadas entre varias de sus 11 fuentes ('Documento' en 8 BD, 'Solicitud' en 8 BD, 'Aporte' en 8 BD, 'Persona' en 8 BD), sin un maestro único consolidado; el 55% de las columnas de esas fuentes está documentado con comentarios.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>'Documento' es la entidad más transversal del dominio (presente en 8 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Solicitud, Aporte para reducir la fragmentación. Debe mejorarse la documentación (55% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Documento, Solicitud, Aporte, Persona, Expediente/Trámite, Beneficiario, Notificación, Recaudación/Pago, Pensión/Pensionista, Planilla, Prestación/Beneficio, Derecho previsional, Resolución, Asegurado/Afiliado, SCTR, Fiscalización, Empleador/Aportante, Inversión/FCR.</t>
         </is>
       </c>
     </row>
@@ -694,12 +694,12 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>El dominio se concentra en 1 fuente, sin fragmentación de entidades entre fuentes. El 45% de las columnas tiene comentarios; conviene mejorar la documentación del dato.</t>
+          <t>Severidad Media (45% documentado): el dominio se concentra en 1 fuente, sin fragmentación de entidades entre fuentes; el 45% de las columnas tiene comentarios.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>La entidad predominante del dominio es 'Documento'. Conviene mejorar la documentación (45% columnas comentadas) para el modelado. Correspondencia con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Documento, Recaudación/Pago, Asegurado/Afiliado, Persona, Solicitud, Expediente/Trámite, Aporte, Empleador/Aportante, Beneficiario, Pensión/Pensionista, Planilla, Resolución, SCTR, Notificación, Derecho previsional, Prestación/Beneficio.</t>
         </is>
       </c>
     </row>
@@ -762,12 +762,12 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Las entidades core del dominio están fragmentadas entre varias de sus 3 fuentes ('Aporte' en 3 BD, 'Persona' en 3 BD, 'Documento' en 3 BD, 'Asegurado/Afiliado' en 3 BD), sin un maestro único consolidado. Además, solo el 22% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
+          <t>Severidad Crítica (22% documentado): las entidades core están fragmentadas entre varias de sus 3 fuentes ('Aporte' en 3 BD, 'Persona' en 3 BD, 'Documento' en 3 BD, 'Asegurado/Afiliado' en 3 BD), sin un maestro único consolidado; el 22% de las columnas de esas fuentes está documentado con comentarios.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>'Aporte' es la entidad más transversal del dominio (presente en 3 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Persona, Documento para reducir la fragmentación. Debe mejorarse la documentación (22% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Aporte, Persona, Documento, Asegurado/Afiliado, Empleador/Aportante, Recaudación/Pago, Pensión/Pensionista, SCTR, Planilla, Inversión/FCR, Expediente/Trámite, Solicitud, Beneficiario, Prestación/Beneficio, Derecho previsional, Notificación, Resolución, Fiscalización.</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Las entidades core del dominio están fragmentadas entre varias de sus 10 fuentes ('Documento' en 9 BD, 'Solicitud' en 9 BD, 'Aporte' en 9 BD, 'Expediente/Trámite' en 9 BD), sin un maestro único consolidado. Además, solo el 40% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
+          <t>Severidad Media (40% documentado): las entidades core están fragmentadas entre varias de sus 10 fuentes ('Documento' en 9 BD, 'Solicitud' en 9 BD, 'Aporte' en 9 BD, 'Expediente/Trámite' en 9 BD), sin un maestro único consolidado; el 40% de las columnas de esas fuentes está documentado con comentarios.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>'Documento' es la entidad más transversal del dominio (presente en 9 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Solicitud, Aporte para reducir la fragmentación. Debe mejorarse la documentación (40% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Documento, Solicitud, Aporte, Expediente/Trámite, Persona, Notificación, Recaudación/Pago, Pensión/Pensionista, Beneficiario, Asegurado/Afiliado, Planilla, Resolución, Derecho previsional, Prestación/Beneficio, SCTR, Fiscalización, Empleador/Aportante, Apelación, Inversión/FCR.</t>
         </is>
       </c>
     </row>
@@ -902,12 +902,12 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Las entidades core del dominio están fragmentadas entre varias de sus 82 fuentes ('Documento' en 21 BD, 'Expediente/Trámite' en 21 BD, 'Persona' en 20 BD, 'Solicitud' en 20 BD), sin un maestro único consolidado. Además, solo el 34% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
+          <t>Severidad Alta (34% documentado): las entidades core están fragmentadas entre varias de sus 82 fuentes ('Documento' en 21 BD, 'Expediente/Trámite' en 21 BD, 'Persona' en 20 BD, 'Solicitud' en 20 BD), sin un maestro único consolidado; el 34% de las columnas de esas fuentes está documentado con comentarios.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>'Documento' es la entidad más transversal del dominio (presente en 21 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Expediente/Trámite, Persona para reducir la fragmentación. Debe mejorarse la documentación (34% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Documento, Expediente/Trámite, Persona, Solicitud, Notificación, Aporte, Pensión/Pensionista, Recaudación/Pago, Empleador/Aportante, Asegurado/Afiliado, Beneficiario, Planilla, Resolución, SCTR, Prestación/Beneficio, Derecho previsional, Fiscalización, Inversión/FCR, Apelación.</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Las entidades core del dominio están fragmentadas entre varias de sus 9 fuentes ('Aporte' en 7 BD, 'Persona' en 7 BD, 'Documento' en 7 BD, 'Asegurado/Afiliado' en 7 BD), sin un maestro único consolidado. Además, solo el 23% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
+          <t>Severidad Alta (23% documentado): las entidades core están fragmentadas entre varias de sus 9 fuentes ('Aporte' en 7 BD, 'Persona' en 7 BD, 'Documento' en 7 BD, 'Asegurado/Afiliado' en 7 BD), sin un maestro único consolidado; el 23% de las columnas de esas fuentes está documentado con comentarios.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>'Aporte' es la entidad más transversal del dominio (presente en 7 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Persona, Documento para reducir la fragmentación. Debe mejorarse la documentación (23% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Aporte, Persona, Documento, Asegurado/Afiliado, Recaudación/Pago, Pensión/Pensionista, Beneficiario, Solicitud, Expediente/Trámite, SCTR, Planilla, Prestación/Beneficio, Derecho previsional, Resolución, Notificación, Fiscalización, Empleador/Aportante, Inversión/FCR.</t>
         </is>
       </c>
     </row>
@@ -1046,12 +1046,12 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Las entidades core del dominio están fragmentadas entre varias de sus 50 fuentes ('Aporte' en 3 BD, 'Documento' en 3 BD, 'Persona' en 3 BD, 'Expediente/Trámite' en 3 BD), sin un maestro único consolidado. Además, solo el 57% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
+          <t>Severidad Mínima (57% documentado): las entidades core están fragmentadas entre varias de sus 50 fuentes ('Aporte' en 3 BD, 'Documento' en 3 BD, 'Persona' en 3 BD, 'Expediente/Trámite' en 3 BD), sin un maestro único consolidado; el 57% de las columnas de esas fuentes está documentado con comentarios.</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>'Aporte' es la entidad más transversal del dominio (presente en 3 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Documento, Persona para reducir la fragmentación. Debe mejorarse la documentación (57% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Aporte, Documento, Persona, Expediente/Trámite, Solicitud, Notificación, Beneficiario, Asegurado/Afiliado, Empleador/Aportante, Planilla, Pensión/Pensionista, Recaudación/Pago, Inversión/FCR, SCTR, Resolución, Prestación/Beneficio, Derecho previsional, Fiscalización.</t>
         </is>
       </c>
     </row>
@@ -1118,12 +1118,12 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Las entidades core del dominio están fragmentadas entre varias de sus 17 fuentes ('Documento' en 9 BD, 'Expediente/Trámite' en 9 BD, 'Notificación' en 9 BD, 'Persona' en 8 BD), sin un maestro único consolidado. Además, solo el 48% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
+          <t>Severidad Baja (48% documentado): las entidades core están fragmentadas entre varias de sus 17 fuentes ('Documento' en 9 BD, 'Expediente/Trámite' en 9 BD, 'Notificación' en 9 BD, 'Persona' en 8 BD), sin un maestro único consolidado; el 48% de las columnas de esas fuentes está documentado con comentarios.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>'Documento' es la entidad más transversal del dominio (presente en 9 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Expediente/Trámite, Notificación para reducir la fragmentación. Debe mejorarse la documentación (48% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Documento, Expediente/Trámite, Notificación, Persona, Solicitud, Aporte, Asegurado/Afiliado, Pensión/Pensionista, Empleador/Aportante, Recaudación/Pago, Beneficiario, Planilla, SCTR, Resolución, Prestación/Beneficio, Fiscalización, Derecho previsional, Inversión/FCR.</t>
         </is>
       </c>
     </row>
@@ -1190,12 +1190,12 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Las entidades core del dominio están fragmentadas entre varias de sus 73 fuentes ('Documento' en 16 BD, 'Aporte' en 15 BD, 'Persona' en 15 BD, 'Solicitud' en 15 BD), sin un maestro único consolidado. Además, solo el 24% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
+          <t>Severidad Alta (24% documentado): las entidades core están fragmentadas entre varias de sus 73 fuentes ('Documento' en 16 BD, 'Aporte' en 15 BD, 'Persona' en 15 BD, 'Solicitud' en 15 BD), sin un maestro único consolidado; el 24% de las columnas de esas fuentes está documentado con comentarios.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>'Documento' es la entidad más transversal del dominio (presente en 16 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Aporte, Persona para reducir la fragmentación. Debe mejorarse la documentación (24% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Documento, Aporte, Persona, Solicitud, Expediente/Trámite, Notificación, Pensión/Pensionista, Recaudación/Pago, SCTR, Beneficiario, Asegurado/Afiliado, Empleador/Aportante, Planilla, Prestación/Beneficio, Resolución, Derecho previsional, Fiscalización, Inversión/FCR, Apelación.</t>
         </is>
       </c>
     </row>
@@ -1238,12 +1238,12 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Sin fuentes de datos asociadas en el inventario: vacío total (no hay sistemas ni BD mapeadas).</t>
+          <t>Severidad Crítica (0% documentado): sin fuentes de datos asociadas en el inventario (vacío total: no hay sistemas ni BD mapeadas).</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Sin entidades detectadas (fuentes sin catálogo o dominio no misional); requiere identificar sus sistemas de soporte para el modelado.</t>
+          <t>No aporta entidades al modelo conceptual (sin estructura catalogada).</t>
         </is>
       </c>
     </row>
@@ -1310,12 +1310,12 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Las entidades core del dominio están fragmentadas entre varias de sus 4 fuentes ('Documento' en 2 BD, 'Persona' en 2 BD, 'Solicitud' en 2 BD, 'Expediente/Trámite' en 2 BD), sin un maestro único consolidado. Además, solo el 46% de las columnas de esas fuentes tiene comentarios, lo que limita el entendimiento y la trazabilidad del dato.</t>
+          <t>Severidad Baja (46% documentado): las entidades core están fragmentadas entre varias de sus 4 fuentes ('Documento' en 2 BD, 'Persona' en 2 BD, 'Solicitud' en 2 BD, 'Expediente/Trámite' en 2 BD), sin un maestro único consolidado; el 46% de las columnas de esas fuentes está documentado con comentarios.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>'Documento' es la entidad más transversal del dominio (presente en 2 fuentes): candidata a entidad maestra única del BDI, a consolidar junto con Persona, Solicitud para reducir la fragmentación. Debe mejorarse la documentación (46% columnas comentadas) de cara al modelado. Correspondencia detallada con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Documento, Persona, Solicitud, Expediente/Trámite, Aporte, Empleador/Aportante, Pensión/Pensionista, Notificación, SCTR, Recaudación/Pago, Asegurado/Afiliado, Beneficiario, Planilla, Resolución, Derecho previsional, Prestación/Beneficio, Fiscalización.</t>
         </is>
       </c>
     </row>
@@ -1378,12 +1378,12 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>De 6 fuentes del dominio, solo 1 con catálogo de entidades documentado (cobertura del modelo parcial). El 81% de las columnas tiene comentarios, por lo que la documentación del dato es limitada.</t>
+          <t>Severidad Mínima (81% documentado): de 6 fuentes del dominio, solo 1 tiene su estructura física catalogada (cobertura del modelo parcial); el 81% de las columnas tiene comentarios.</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>La entidad predominante del dominio es 'Aporte'. Conviene ampliar el catálogo de las 5 fuentes sin documentar para el modelado. Correspondencia con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Aporte, Asegurado/Afiliado, Documento, Planilla, Persona, Empleador/Aportante, Inversión/FCR, Solicitud, Recaudación/Pago, SCTR, Pensión/Pensionista, Beneficiario, Derecho previsional, Prestación/Beneficio, Notificación, Expediente/Trámite.</t>
         </is>
       </c>
     </row>
@@ -1446,12 +1446,12 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>El dominio se concentra en 1 fuente, sin fragmentación de entidades entre fuentes. El 66% de las columnas tiene comentarios; conviene mejorar la documentación del dato.</t>
+          <t>Severidad Mínima (66% documentado): el dominio se concentra en 1 fuente, sin fragmentación de entidades entre fuentes; el 66% de las columnas tiene comentarios.</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>La entidad predominante del dominio es 'Documento'. Conviene mejorar la documentación (66% columnas comentadas) para el modelado. Correspondencia con el SIIP pendiente (dominios de datos no definidos en el MC).</t>
+          <t>Entidades que aporta al modelo conceptual: Documento, Recaudación/Pago, Expediente/Trámite, Persona, Notificación, Solicitud, Resolución, Pensión/Pensionista, Apelación, Aporte, Beneficiario, Empleador/Aportante.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ADI-04: Vacíos/dispersión con texto humano por severidad + indicador de dispersión (favorable↔desfavorable)
- Documentación: frase según severidad (muy deficiente/escasa/parcial/aceptable/adecuada) mostrando el %
- Dispersión: indicador (baja favorable / moderada / alta / muy alta desfavorable, con 'hasta N BD' y
  recomendación de maestro único); 'no evaluable' cuando la cobertura de catálogo es insuficiente

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client/public/artefactos/ADI-04.xlsx
+++ b/client/public/artefactos/ADI-04.xlsx
@@ -558,7 +558,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Severidad Crítica (15% documentado): de 26 fuentes del dominio, solo 1 tiene su estructura física catalogada (cobertura del modelo parcial); el 15% de las columnas tiene comentarios.</t>
+          <t>Dispersión no evaluable con la cobertura actual: solo 1 de 26 fuentes tiene estructura física catalogada. La documentación del dato es muy deficiente (15% de columnas comentadas), lo que impide entenderlo sin apoyo del gestor.</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Severidad Baja (55% documentado): las entidades core están fragmentadas entre varias de sus 11 fuentes ('Documento' en 8 BD, 'Solicitud' en 8 BD, 'Aporte' en 8 BD, 'Persona' en 8 BD), sin un maestro único consolidado; el 55% de las columnas de esas fuentes está documentado con comentarios.</t>
+          <t>Dispersión muy alta: entidades como 'Documento', 'Solicitud', 'Aporte' están presentes en varias fuentes (hasta 8 BD), evidenciando fragmentación sin un maestro consolidado — situación desfavorable que justifica consolidar un maestro único en el BDI. La documentación del dato es aceptable (55% de columnas comentadas), aunque mejorable.</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Severidad Media (45% documentado): el dominio se concentra en 1 fuente, sin fragmentación de entidades entre fuentes; el 45% de las columnas tiene comentarios.</t>
+          <t>Dispersión baja (favorable): la información se concentra en 1 fuente, sin fragmentación entre fuentes. La documentación del dato es parcial (45% de columnas comentadas); conviene completarla.</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -762,7 +762,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Severidad Crítica (22% documentado): las entidades core están fragmentadas entre varias de sus 3 fuentes ('Aporte' en 3 BD, 'Persona' en 3 BD, 'Documento' en 3 BD, 'Asegurado/Afiliado' en 3 BD), sin un maestro único consolidado; el 22% de las columnas de esas fuentes está documentado con comentarios.</t>
+          <t>Dispersión moderada: entidades como 'Aporte', 'Persona', 'Documento' están presentes en varias fuentes (hasta 3 BD), evidenciando fragmentación sin un maestro consolidado, lo que invita a evaluar un maestro único. La documentación del dato es muy deficiente (22% de columnas comentadas), lo que impide entenderlo sin apoyo del gestor.</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -830,7 +830,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Severidad Media (40% documentado): las entidades core están fragmentadas entre varias de sus 10 fuentes ('Documento' en 9 BD, 'Solicitud' en 9 BD, 'Aporte' en 9 BD, 'Expediente/Trámite' en 9 BD), sin un maestro único consolidado; el 40% de las columnas de esas fuentes está documentado con comentarios.</t>
+          <t>Dispersión muy alta: entidades como 'Documento', 'Solicitud', 'Aporte' están presentes en varias fuentes (hasta 9 BD), evidenciando fragmentación sin un maestro consolidado — situación desfavorable que justifica consolidar un maestro único en el BDI. La documentación del dato es parcial (40% de columnas comentadas); conviene completarla.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -902,7 +902,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Severidad Alta (34% documentado): las entidades core están fragmentadas entre varias de sus 82 fuentes ('Documento' en 21 BD, 'Expediente/Trámite' en 21 BD, 'Persona' en 20 BD, 'Solicitud' en 20 BD), sin un maestro único consolidado; el 34% de las columnas de esas fuentes está documentado con comentarios.</t>
+          <t>Dispersión muy alta: entidades como 'Documento', 'Expediente/Trámite', 'Persona' están presentes en varias fuentes (hasta 21 BD), evidenciando fragmentación sin un maestro consolidado — situación desfavorable que justifica consolidar un maestro único en el BDI. La documentación del dato es escasa (34% de columnas comentadas), lo que limita su entendimiento.</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -974,7 +974,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Severidad Alta (23% documentado): las entidades core están fragmentadas entre varias de sus 9 fuentes ('Aporte' en 7 BD, 'Persona' en 7 BD, 'Documento' en 7 BD, 'Asegurado/Afiliado' en 7 BD), sin un maestro único consolidado; el 23% de las columnas de esas fuentes está documentado con comentarios.</t>
+          <t>Dispersión alta: entidades como 'Aporte', 'Persona', 'Documento' están presentes en varias fuentes (hasta 7 BD), evidenciando fragmentación sin un maestro consolidado — situación desfavorable que justifica consolidar un maestro único en el BDI. La documentación del dato es escasa (23% de columnas comentadas), lo que limita su entendimiento.</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Severidad Mínima (57% documentado): las entidades core están fragmentadas entre varias de sus 50 fuentes ('Aporte' en 3 BD, 'Documento' en 3 BD, 'Persona' en 3 BD, 'Expediente/Trámite' en 3 BD), sin un maestro único consolidado; el 57% de las columnas de esas fuentes está documentado con comentarios.</t>
+          <t>Dispersión moderada: entidades como 'Aporte', 'Documento', 'Persona' están presentes en varias fuentes (hasta 3 BD), evidenciando fragmentación sin un maestro consolidado, lo que invita a evaluar un maestro único. La documentación del dato es adecuada (57% de columnas comentadas).</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Severidad Baja (48% documentado): las entidades core están fragmentadas entre varias de sus 17 fuentes ('Documento' en 9 BD, 'Expediente/Trámite' en 9 BD, 'Notificación' en 9 BD, 'Persona' en 8 BD), sin un maestro único consolidado; el 48% de las columnas de esas fuentes está documentado con comentarios.</t>
+          <t>Dispersión muy alta: entidades como 'Documento', 'Expediente/Trámite', 'Notificación' están presentes en varias fuentes (hasta 9 BD), evidenciando fragmentación sin un maestro consolidado — situación desfavorable que justifica consolidar un maestro único en el BDI. La documentación del dato es aceptable (48% de columnas comentadas), aunque mejorable.</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1190,7 +1190,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Severidad Alta (24% documentado): las entidades core están fragmentadas entre varias de sus 73 fuentes ('Documento' en 16 BD, 'Aporte' en 15 BD, 'Persona' en 15 BD, 'Solicitud' en 15 BD), sin un maestro único consolidado; el 24% de las columnas de esas fuentes está documentado con comentarios.</t>
+          <t>Dispersión muy alta: entidades como 'Documento', 'Aporte', 'Persona' están presentes en varias fuentes (hasta 16 BD), evidenciando fragmentación sin un maestro consolidado — situación desfavorable que justifica consolidar un maestro único en el BDI. La documentación del dato es escasa (24% de columnas comentadas), lo que limita su entendimiento.</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1238,7 +1238,7 @@
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Severidad Crítica (0% documentado): sin fuentes de datos asociadas en el inventario (vacío total: no hay sistemas ni BD mapeadas).</t>
+          <t>Sin fuentes de datos asociadas en el inventario (vacío total: no hay sistemas ni BD mapeadas).</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Severidad Baja (46% documentado): las entidades core están fragmentadas entre varias de sus 4 fuentes ('Documento' en 2 BD, 'Persona' en 2 BD, 'Solicitud' en 2 BD, 'Expediente/Trámite' en 2 BD), sin un maestro único consolidado; el 46% de las columnas de esas fuentes está documentado con comentarios.</t>
+          <t>Dispersión moderada: entidades como 'Documento', 'Persona', 'Solicitud' están presentes en varias fuentes (hasta 2 BD), evidenciando fragmentación sin un maestro consolidado, lo que invita a evaluar un maestro único. La documentación del dato es aceptable (46% de columnas comentadas), aunque mejorable.</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Severidad Mínima (81% documentado): de 6 fuentes del dominio, solo 1 tiene su estructura física catalogada (cobertura del modelo parcial); el 81% de las columnas tiene comentarios.</t>
+          <t>Dispersión no evaluable con la cobertura actual: solo 1 de 6 fuentes tiene estructura física catalogada. La documentación del dato es adecuada (81% de columnas comentadas).</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Severidad Mínima (66% documentado): el dominio se concentra en 1 fuente, sin fragmentación de entidades entre fuentes; el 66% de las columnas tiene comentarios.</t>
+          <t>Dispersión baja (favorable): la información se concentra en 1 fuente, sin fragmentación entre fuentes. La documentación del dato es adecuada (66% de columnas comentadas).</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">

</xml_diff>